<commit_message>
paper run 2026-09-25 11:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-25.xlsx
+++ b/reports/2026-09-25.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -724,13 +724,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>246.69</v>
+        <v>214.21</v>
       </c>
       <c r="E15" t="n">
         <v>3.9</v>
@@ -743,13 +743,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>118.78</v>
+        <v>329.92</v>
       </c>
       <c r="E16" t="n">
         <v>10.8</v>
@@ -765,26 +765,26 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>149.36</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="E18" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -794,433 +794,452 @@
         <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>216.11</v>
+        <v>218.87</v>
       </c>
       <c r="E19" t="n">
-        <v>10.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>258.97</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" t="n">
-        <v>66.2</v>
-      </c>
-      <c r="E21" t="n">
-        <v>10.8</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>158.6</v>
+        <v>277.34</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C23" t="n">
         <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>140.67</v>
+        <v>84.92</v>
       </c>
       <c r="E23" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>181.87</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>5</v>
-      </c>
-      <c r="C25" t="n">
-        <v>5</v>
-      </c>
-      <c r="D25" t="n">
-        <v>251.46</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>10</v>
+      </c>
+      <c r="C26" t="n">
+        <v>9</v>
+      </c>
+      <c r="D26" t="n">
+        <v>430.12</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B27" t="n">
         <v>2</v>
       </c>
-      <c r="C26" t="n">
+      <c r="C27" t="n">
         <v>2</v>
       </c>
-      <c r="D26" t="n">
+      <c r="D27" t="n">
         <v>114.01</v>
       </c>
-      <c r="E26" t="n">
+      <c r="E27" t="n">
         <v>14.7</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>3.9</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>XRP</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
         <v>10.8</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="n">
-        <v>3.9</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
         <v>10.8</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>00</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
-        <v>10.8</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
         <v>3.9</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" t="n">
-        <v>10.8</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>0.60–0.62</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" t="n">
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
         <v>3.9</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" t="n">
-        <v>10.8</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>0.15–0.20%</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="n">
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
         <v>3.9</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B52" t="n">
         <v>2</v>
       </c>
-      <c r="C51" t="n">
+      <c r="C52" t="n">
         <v>2</v>
       </c>
-      <c r="D51" t="n">
+      <c r="D52" t="n">
         <v>14.7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-09-25 17:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-25.xlsx
+++ b/reports/2026-09-25.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,307 @@
       </c>
       <c r="K3" t="n">
         <v>3.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-25T12:27:31.867582+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F4" t="n">
+        <v>84.95999999999999</v>
+      </c>
+      <c r="G4" t="n">
+        <v>154.47</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00119</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>69.51000000000001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-25T13:12:44.665869+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F5" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="G5" t="n">
+        <v>44.17</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00112</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>20.32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-25T13:57:17.491580+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F6" t="n">
+        <v>13.54</v>
+      </c>
+      <c r="G6" t="n">
+        <v>25.08</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.8090000000000001</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.00211</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>11.54</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-25T14:18:52.717117+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00134</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-25T15:03:56.583793+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5223</v>
+      </c>
+      <c r="F8" t="n">
+        <v>65.59</v>
+      </c>
+      <c r="G8" t="n">
+        <v>125.58</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.783</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.00157</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-25T15:18:53.505797+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F9" t="n">
+        <v>30.23</v>
+      </c>
+      <c r="G9" t="n">
+        <v>48.76</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0.00138</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>18.53</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-25T17:08:46.667619+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.4544</v>
+      </c>
+      <c r="F10" t="n">
+        <v>18.63</v>
+      </c>
+      <c r="G10" t="n">
+        <v>41</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-0.00137</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>-18.63</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +894,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +904,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -613,7 +914,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -623,7 +924,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +934,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14.7</v>
+        <v>178.31</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +944,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14.7</v>
+        <v>196.94</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +954,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-18.63</v>
       </c>
     </row>
     <row r="9">
@@ -663,7 +964,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>10.57</v>
       </c>
     </row>
     <row r="10">
@@ -673,7 +974,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1699.220000000001</v>
+        <v>1862.830000000001</v>
       </c>
     </row>
     <row r="12">
@@ -724,16 +1025,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>214.21</v>
+        <v>327.37</v>
       </c>
       <c r="E15" t="n">
-        <v>3.9</v>
+        <v>105.27</v>
       </c>
     </row>
     <row r="16">
@@ -743,16 +1044,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D16" t="n">
-        <v>329.92</v>
+        <v>855.01</v>
       </c>
       <c r="E16" t="n">
-        <v>10.8</v>
+        <v>73.04000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -765,7 +1066,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -775,354 +1076,370 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>66.29000000000001</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>69.51000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
         <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>218.87</v>
+        <v>176.2</v>
       </c>
       <c r="E19" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C20" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D20" t="n">
-        <v>258.97</v>
+        <v>591.92</v>
       </c>
       <c r="E20" t="n">
-        <v>10.8</v>
+        <v>26.57</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>18</v>
+      </c>
+      <c r="C21" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" t="n">
+        <v>344.75</v>
+      </c>
+      <c r="E21" t="n">
+        <v>82.23</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>4</v>
-      </c>
-      <c r="C22" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" t="n">
-        <v>277.34</v>
-      </c>
-      <c r="E22" t="n">
-        <v>10.8</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D23" t="n">
-        <v>84.92</v>
+        <v>594.51</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>155.88</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D24" t="n">
-        <v>181.87</v>
+        <v>282.52</v>
       </c>
       <c r="E24" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>9</v>
+      </c>
+      <c r="C25" t="n">
+        <v>8</v>
+      </c>
+      <c r="D25" t="n">
+        <v>305.35</v>
+      </c>
+      <c r="E25" t="n">
+        <v>22.43</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>10</v>
-      </c>
-      <c r="C26" t="n">
-        <v>9</v>
-      </c>
-      <c r="D26" t="n">
-        <v>430.12</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>114.01</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>14.7</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>26</v>
+      </c>
+      <c r="C28" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" t="n">
+        <v>662.11</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>9</v>
+      </c>
+      <c r="C29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" t="n">
+        <v>450.76</v>
+      </c>
+      <c r="E29" t="n">
+        <v>178.31</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>3.9</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
         <v>1</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C34" t="n">
         <v>1</v>
       </c>
-      <c r="D33" t="n">
-        <v>10.8</v>
+      <c r="D34" t="n">
+        <v>69.51000000000001</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="n">
+        <v>26.57</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>10.8</v>
+        <v>82.23</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" t="n">
+        <v>105.27</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>00</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D40" t="n">
-        <v>10.8</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>3.9</v>
+        <v>73.04000000000001</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>10.8</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1132,13 +1449,13 @@
         <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>10.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1148,67 +1465,77 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>3.9</v>
+        <v>69.51000000000001</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>31.86</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.35</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>10.8</v>
+        <v>78.52</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>3.9</v>
+        <v>-18.63</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>По направлению</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1230,17 +1557,173 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>7</v>
+      </c>
+      <c r="C52" t="n">
+        <v>6</v>
+      </c>
+      <c r="D52" t="n">
+        <v>155.88</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" t="n">
+        <v>22.43</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" t="n">
+        <v>100.63</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
+        <v>63.89</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>11.54</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" t="n">
+        <v>71.43000000000001</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B52" t="n">
-        <v>2</v>
-      </c>
-      <c r="C52" t="n">
-        <v>2</v>
-      </c>
-      <c r="D52" t="n">
-        <v>14.7</v>
+      <c r="B63" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D63" t="n">
+        <v>106.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-25 23:53
</commit_message>
<xml_diff>
--- a/reports/2026-09-25.xlsx
+++ b/reports/2026-09-25.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -859,6 +859,49 @@
       </c>
       <c r="K10" t="n">
         <v>-18.63</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-25T19:13:49.290287+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F11" t="n">
+        <v>14.56</v>
+      </c>
+      <c r="G11" t="n">
+        <v>26</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>11.44</v>
       </c>
     </row>
   </sheetData>
@@ -872,7 +915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,7 +937,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -904,7 +947,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -924,7 +967,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="6">
@@ -934,7 +977,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>178.31</v>
+        <v>189.75</v>
       </c>
     </row>
     <row r="7">
@@ -944,7 +987,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>196.94</v>
+        <v>208.38</v>
       </c>
     </row>
     <row r="8">
@@ -964,7 +1007,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10.57</v>
+        <v>11.19</v>
       </c>
     </row>
     <row r="10">
@@ -974,7 +1017,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1862.830000000001</v>
+        <v>1874.270000000001</v>
       </c>
     </row>
     <row r="12">
@@ -1025,13 +1068,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D15" t="n">
-        <v>327.37</v>
+        <v>374.38</v>
       </c>
       <c r="E15" t="n">
         <v>105.27</v>
@@ -1044,16 +1087,16 @@
         </is>
       </c>
       <c r="B16" t="n">
+        <v>17</v>
+      </c>
+      <c r="C16" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="n">
-        <v>14</v>
-      </c>
       <c r="D16" t="n">
-        <v>855.01</v>
+        <v>834.48</v>
       </c>
       <c r="E16" t="n">
-        <v>73.04000000000001</v>
+        <v>84.48</v>
       </c>
     </row>
     <row r="17">
@@ -1108,16 +1151,16 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>13</v>
+      </c>
+      <c r="C20" t="n">
         <v>12</v>
       </c>
-      <c r="C20" t="n">
-        <v>11</v>
-      </c>
       <c r="D20" t="n">
-        <v>591.92</v>
+        <v>665.1</v>
       </c>
       <c r="E20" t="n">
-        <v>26.57</v>
+        <v>38.01</v>
       </c>
     </row>
     <row r="21">
@@ -1127,13 +1170,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D21" t="n">
-        <v>344.75</v>
+        <v>298.05</v>
       </c>
       <c r="E21" t="n">
         <v>82.23</v>
@@ -1153,13 +1196,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C23" t="n">
         <v>13</v>
       </c>
       <c r="D23" t="n">
-        <v>594.51</v>
+        <v>500.8</v>
       </c>
       <c r="E23" t="n">
         <v>155.88</v>
@@ -1172,16 +1215,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>282.52</v>
+        <v>355.7</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>11.44</v>
       </c>
     </row>
     <row r="25">
@@ -1191,13 +1234,13 @@
         </is>
       </c>
       <c r="B25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" t="n">
         <v>9</v>
       </c>
-      <c r="C25" t="n">
-        <v>8</v>
-      </c>
       <c r="D25" t="n">
-        <v>305.35</v>
+        <v>352.36</v>
       </c>
       <c r="E25" t="n">
         <v>22.43</v>
@@ -1236,13 +1279,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C28" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D28" t="n">
-        <v>662.11</v>
+        <v>615.41</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1255,16 +1298,16 @@
         </is>
       </c>
       <c r="B29" t="n">
+        <v>10</v>
+      </c>
+      <c r="C29" t="n">
         <v>9</v>
       </c>
-      <c r="C29" t="n">
-        <v>8</v>
-      </c>
       <c r="D29" t="n">
-        <v>450.76</v>
+        <v>523.9400000000001</v>
       </c>
       <c r="E29" t="n">
-        <v>178.31</v>
+        <v>189.75</v>
       </c>
     </row>
     <row r="31">
@@ -1319,13 +1362,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>26.57</v>
+        <v>38.01</v>
       </c>
     </row>
     <row r="36">
@@ -1389,13 +1432,13 @@
         </is>
       </c>
       <c r="B40" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" t="n">
         <v>5</v>
       </c>
-      <c r="C40" t="n">
-        <v>4</v>
-      </c>
       <c r="D40" t="n">
-        <v>73.04000000000001</v>
+        <v>84.48</v>
       </c>
     </row>
     <row r="42">
@@ -1532,198 +1575,230 @@
         <v>-18.63</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>11.44</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>7</v>
-      </c>
-      <c r="C52" t="n">
-        <v>6</v>
-      </c>
-      <c r="D52" t="n">
-        <v>155.88</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D53" t="n">
-        <v>22.43</v>
+        <v>155.88</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>11.44</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>3</v>
-      </c>
-      <c r="C56" t="n">
-        <v>3</v>
-      </c>
-      <c r="D56" t="n">
-        <v>100.63</v>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>22.43</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>3</v>
-      </c>
-      <c r="C57" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" t="n">
-        <v>2.25</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D58" t="n">
-        <v>63.89</v>
+        <v>100.63</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0.20%+</t>
+          <t>0.12–0.15%</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
-        <v>11.54</v>
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" t="n">
+        <v>63.89</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>4</v>
-      </c>
-      <c r="C62" t="n">
-        <v>3</v>
-      </c>
-      <c r="D62" t="n">
-        <v>71.43000000000001</v>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" t="n">
+        <v>22.98</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>4</v>
+      </c>
+      <c r="C64" t="n">
+        <v>3</v>
+      </c>
+      <c r="D64" t="n">
+        <v>71.43000000000001</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B63" t="n">
-        <v>5</v>
-      </c>
-      <c r="C63" t="n">
-        <v>5</v>
-      </c>
-      <c r="D63" t="n">
-        <v>106.88</v>
+      <c r="B65" t="n">
+        <v>6</v>
+      </c>
+      <c r="C65" t="n">
+        <v>6</v>
+      </c>
+      <c r="D65" t="n">
+        <v>118.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>